<commit_message>
deployment to streamlit cloud
</commit_message>
<xml_diff>
--- a/src/data/Template.xlsx
+++ b/src/data/Template.xlsx
@@ -1,203 +1,267 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="12180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView windowWidth="10668" windowHeight="6132"/>
   </bookViews>
   <sheets>
-    <sheet name="Variables template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Análisis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Variables template" sheetId="1" r:id="rId1"/>
+    <sheet name="Análisis" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Fecha de venta</t>
+  </si>
+  <si>
+    <t>Accion</t>
+  </si>
+  <si>
+    <t>Producto</t>
+  </si>
+  <si>
+    <t>Botellas vendidas</t>
+  </si>
+  <si>
+    <t>Precio total venta</t>
+  </si>
+  <si>
+    <t>Precio botella</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Metodo de pago</t>
+  </si>
+  <si>
+    <t>Análisis a incluir</t>
+  </si>
+  <si>
+    <t>Volumen de stock</t>
+  </si>
+  <si>
+    <t>Stock etiquetado</t>
+  </si>
+  <si>
+    <t>Stock sin etiquetar</t>
+  </si>
+  <si>
+    <t>Ventas por tipología de cliente</t>
+  </si>
+  <si>
+    <t>Precio medio de venta botella</t>
+  </si>
+  <si>
+    <t>Beneficio por método de pago</t>
+  </si>
+  <si>
+    <t>Recaudación total, diferenciando el efectivo del bizzum(partiendo de los gastos iniciales )</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* \-??\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0\ &quot;€&quot;_-;\-* #,##0\ &quot;€&quot;_-;_-* &quot;-&quot;\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="6">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* \-??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0\ &quot;€&quot;_-;\-* #,##0\ &quot;€&quot;_-;_-* &quot;-&quot;\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="179" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <color theme="0"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="37">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -413,7 +477,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -534,178 +598,165 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -759,74 +810,11 @@
     <cellStyle name="60% - Énfasis6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1026,309 +1014,111 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Fecha de venta</t>
-        </is>
+    <row r="1" spans="1:9">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Accion</t>
-        </is>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
       </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>Producto</t>
-        </is>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
       </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>Botellas vendidas</t>
-        </is>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
       </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
-          <t>Precio total venta</t>
-        </is>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
       </c>
-      <c r="F1" s="8" t="inlineStr">
-        <is>
-          <t>Precio botella</t>
-        </is>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
       </c>
-      <c r="G1" s="8" t="inlineStr">
-        <is>
-          <t>Cliente</t>
-        </is>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="H1" s="8" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
       </c>
-      <c r="I1" s="8" t="inlineStr">
-        <is>
-          <t>Metodo de pago</t>
-        </is>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="12" t="n">
-        <v>45690</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sembra 2023</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F2" t="n">
-        <v>50</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Distribución</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
+    <row r="2" spans="1:1">
+      <c r="A2" s="6"/>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="n">
-        <v>45690</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>sembra 2023</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Horeca</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
+    <row r="3" spans="1:1">
+      <c r="A3" s="6"/>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="n">
-        <v>45690</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>sembra 2023</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F4" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Amigos/Familia</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Bizum</t>
-        </is>
-      </c>
+    <row r="4" spans="1:1">
+      <c r="A4" s="6"/>
     </row>
-    <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>45690</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>sembra 2023</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>20</v>
-      </c>
-      <c r="F5" t="n">
-        <v>6.67</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Amigos/Familia</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Bizum</t>
-        </is>
-      </c>
+    <row r="5" spans="1:1">
+      <c r="A5" s="6"/>
     </row>
-    <row r="6">
-      <c r="A6" s="11" t="n">
-        <v>45691</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>sembra 2023</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="n">
-        <v>50</v>
-      </c>
-      <c r="F6" t="n">
-        <v>16.67</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Horeca</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Factura</t>
-        </is>
-      </c>
+    <row r="6" spans="1:1">
+      <c r="A6" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor theme="6"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:A1000"/>
+  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="76.5714285714286" customWidth="1" min="1" max="1"/>
-    <col width="9.142857142857141" customWidth="1" min="2" max="26"/>
+    <col min="1" max="1" width="76.5740740740741" customWidth="1"/>
+    <col min="2" max="26" width="9.13888888888889" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Análisis a incluir</t>
-        </is>
+    <row r="1" ht="14.4" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Volumen de stock</t>
-        </is>
+    <row r="2" ht="14.4" spans="1:1">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Stock etiquetado</t>
-        </is>
+    <row r="3" ht="14.4" spans="1:1">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Stock sin etiquetar</t>
-        </is>
+    <row r="4" ht="14.4" spans="1:1">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Ventas por tipología de cliente</t>
-        </is>
+    <row r="5" ht="14.4" spans="1:1">
+      <c r="A5" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Precio medio de venta botella</t>
-        </is>
+    <row r="6" ht="14.4" spans="1:1">
+      <c r="A6" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Beneficio por método de pago</t>
-        </is>
+    <row r="7" ht="14.4" spans="1:1">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Recaudación total, diferenciando el efectivo del bizzum(partiendo de los gastos iniciales )</t>
-        </is>
+    <row r="8" ht="14.4" spans="1:1">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -2313,6 +2103,7 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="1"/>
+  <pageSetup paperSize="1" orientation="landscape"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>